<commit_message>
start Interp F Cattle slurry
Started on interpolation and integration script for field cattle slurry

imported the data, created a compact dict with valve_dfs as values

notice odd behaviour with TIME_NORM_LOCAL collum
</commit_message>
<xml_diff>
--- a/Lab-trails/2026-01-06-cattle-slurry/2026-01-06-cattle-slurry-Picarro.xlsx
+++ b/Lab-trails/2026-01-06-cattle-slurry/2026-01-06-cattle-slurry-Picarro.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29426"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29530"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\mikae\Desktop\Github - speciale\Larsen-2025-Masterthesis-DFCs\Lab-trails\2026-01-06-cattle-slurry\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2C6AA35B-67AE-4852-A776-C6634DBB2106}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3E7A5DA6-C006-43C7-9BF5-9739F73E2725}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-38520" yWindow="-2820" windowWidth="38640" windowHeight="21120" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="360" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Jar and valve id overview" sheetId="1" r:id="rId1"/>
@@ -51,7 +51,7 @@
     Delayed by excacly 1 h from real time</t>
       </text>
     </comment>
-    <comment ref="H8" authorId="1" shapeId="0" xr:uid="{D6A11C27-28E7-4435-BC4A-E3E1711C9750}">
+    <comment ref="I8" authorId="1" shapeId="0" xr:uid="{D6A11C27-28E7-4435-BC4A-E3E1711C9750}">
       <text>
         <t>[Threaded comment]
 Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
@@ -64,7 +64,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="50" uniqueCount="24">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="52" uniqueCount="26">
   <si>
     <t>Picarro ID</t>
   </si>
@@ -136,6 +136,12 @@
   </si>
   <si>
     <t>endtime Piccarro</t>
+  </si>
+  <si>
+    <t>enddate</t>
+  </si>
+  <si>
+    <t>startdate</t>
   </si>
 </sst>
 </file>
@@ -145,19 +151,13 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="0.000"/>
   </numFmts>
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="1" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="9"/>
-      <color indexed="81"/>
-      <name val="Tahoma"/>
-      <family val="2"/>
     </font>
   </fonts>
   <fills count="4">
@@ -192,12 +192,13 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="20" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -487,7 +488,7 @@
   <threadedComment ref="F2" dT="2026-01-08T09:15:27.58" personId="{665E6C45-FDD8-469A-93B0-28134F14276F}" id="{DFE91DE2-97B6-4683-BB64-BFCD2C85D76D}">
     <text>Delayed by excacly 1 h from real time</text>
   </threadedComment>
-  <threadedComment ref="H8" dT="2026-01-08T09:23:24.74" personId="{665E6C45-FDD8-469A-93B0-28134F14276F}" id="{D6A11C27-28E7-4435-BC4A-E3E1711C9750}">
+  <threadedComment ref="I8" dT="2026-01-08T09:23:24.74" personId="{665E6C45-FDD8-469A-93B0-28134F14276F}" id="{D6A11C27-28E7-4435-BC4A-E3E1711C9750}">
     <text>Didn’t write this, using an average from other jar measurements</text>
   </threadedComment>
 </ThreadedComments>
@@ -728,7 +729,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0B1A1D03-873D-49A4-B894-14582A5CC970}">
-  <dimension ref="A1:K25"/>
+  <dimension ref="A1:M25"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="10.44140625" bestFit="1" customWidth="1"/>
@@ -736,14 +737,15 @@
     <col min="3" max="4" width="11" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="11.6640625" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="15.5546875" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="22.21875" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="11.109375" customWidth="1"/>
     <col min="8" max="8" width="21.77734375" bestFit="1" customWidth="1"/>
     <col min="9" max="10" width="21.6640625" bestFit="1" customWidth="1"/>
     <col min="11" max="11" width="15.6640625" bestFit="1" customWidth="1"/>
     <col min="12" max="12" width="23.77734375" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="10.33203125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>5</v>
       </c>
@@ -763,22 +765,28 @@
         <v>9</v>
       </c>
       <c r="G1" t="s">
+        <v>25</v>
+      </c>
+      <c r="H1" t="s">
         <v>20</v>
       </c>
-      <c r="H1" t="s">
+      <c r="I1" t="s">
         <v>21</v>
       </c>
-      <c r="I1" t="s">
+      <c r="J1" t="s">
         <v>10</v>
       </c>
-      <c r="J1" t="s">
+      <c r="K1" t="s">
         <v>22</v>
       </c>
-      <c r="K1" t="s">
+      <c r="L1" t="s">
         <v>23</v>
       </c>
-    </row>
-    <row r="2" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="M1" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="2" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A2">
         <v>1</v>
       </c>
@@ -797,14 +805,29 @@
       <c r="F2" s="1">
         <v>0.42916666666666664</v>
       </c>
-      <c r="G2">
+      <c r="G2" s="5">
+        <v>46028</v>
+      </c>
+      <c r="H2">
         <v>0.22500000000000001</v>
       </c>
-      <c r="H2">
+      <c r="I2">
         <v>0.93799999999999994</v>
       </c>
-    </row>
-    <row r="3" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="J2">
+        <v>0.27400000000000002</v>
+      </c>
+      <c r="K2">
+        <v>0.89700000000000002</v>
+      </c>
+      <c r="L2" s="1">
+        <v>0.54861111111111116</v>
+      </c>
+      <c r="M2" s="5">
+        <v>46034</v>
+      </c>
+    </row>
+    <row r="3" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A3">
         <v>2</v>
       </c>
@@ -820,14 +843,20 @@
       <c r="E3">
         <v>2.1349999999999998</v>
       </c>
-      <c r="G3">
+      <c r="H3">
         <v>0.224</v>
       </c>
-      <c r="H3">
+      <c r="I3">
         <v>0.94399999999999995</v>
       </c>
-    </row>
-    <row r="4" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="J3">
+        <v>0.23300000000000001</v>
+      </c>
+      <c r="K3">
+        <v>0.93799999999999994</v>
+      </c>
+    </row>
+    <row r="4" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A4">
         <v>3</v>
       </c>
@@ -843,14 +872,20 @@
       <c r="E4">
         <v>2.0219999999999998</v>
       </c>
-      <c r="G4">
+      <c r="H4">
         <v>0.22600000000000001</v>
       </c>
-      <c r="H4" s="4">
+      <c r="I4" s="4">
         <v>0.94</v>
       </c>
-    </row>
-    <row r="5" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="J4">
+        <v>0.22900000000000001</v>
+      </c>
+      <c r="K4">
+        <v>0.94099999999999995</v>
+      </c>
+    </row>
+    <row r="5" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A5">
         <v>4</v>
       </c>
@@ -866,14 +901,20 @@
       <c r="E5">
         <v>2.0499999999999998</v>
       </c>
-      <c r="G5">
+      <c r="H5">
         <v>0.22600000000000001</v>
       </c>
-      <c r="H5">
+      <c r="I5">
         <v>0.94499999999999995</v>
       </c>
-    </row>
-    <row r="6" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="J5">
+        <v>0.23599999999999999</v>
+      </c>
+      <c r="K5">
+        <v>0.93400000000000005</v>
+      </c>
+    </row>
+    <row r="6" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A6">
         <v>5</v>
       </c>
@@ -889,14 +930,20 @@
       <c r="E6">
         <v>2.097</v>
       </c>
-      <c r="G6">
+      <c r="H6">
         <v>0.22600000000000001</v>
       </c>
-      <c r="H6">
+      <c r="I6">
         <v>0.94799999999999995</v>
       </c>
-    </row>
-    <row r="7" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="J6">
+        <v>0.23300000000000001</v>
+      </c>
+      <c r="K6">
+        <v>0.93799999999999994</v>
+      </c>
+    </row>
+    <row r="7" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A7">
         <v>11</v>
       </c>
@@ -909,14 +956,20 @@
       <c r="D7" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="G7" s="4">
+      <c r="H7" s="4">
         <v>0.4</v>
       </c>
-      <c r="H7">
+      <c r="I7">
         <v>0.77600000000000002</v>
       </c>
-    </row>
-    <row r="8" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="J7">
+        <v>0.41899999999999998</v>
+      </c>
+      <c r="K7">
+        <v>0.75900000000000001</v>
+      </c>
+    </row>
+    <row r="8" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A8">
         <v>6</v>
       </c>
@@ -932,15 +985,21 @@
       <c r="E8">
         <v>2.0710000000000002</v>
       </c>
-      <c r="G8">
+      <c r="H8">
         <v>0.22700000000000001</v>
       </c>
-      <c r="H8" s="4">
-        <f>AVERAGE(H2:H6,H10:H12,H14:H18,H20:H24)</f>
+      <c r="I8" s="4">
+        <f>AVERAGE(I2:I6,I10:I12,I14:I18,I20:I24)</f>
         <v>0.9454999999999999</v>
       </c>
-    </row>
-    <row r="9" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="J8">
+        <v>0.23400000000000001</v>
+      </c>
+      <c r="K8">
+        <v>0.93600000000000005</v>
+      </c>
+    </row>
+    <row r="9" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A9">
         <v>7</v>
       </c>
@@ -956,14 +1015,20 @@
       <c r="E9">
         <v>2.0819999999999999</v>
       </c>
-      <c r="G9">
+      <c r="H9">
         <v>0.22500000000000001</v>
       </c>
-      <c r="H9">
+      <c r="I9">
         <v>0.94499999999999995</v>
       </c>
-    </row>
-    <row r="10" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="J9" s="4">
+        <v>0.23100000000000001</v>
+      </c>
+      <c r="K9">
+        <v>0.93799999999999994</v>
+      </c>
+    </row>
+    <row r="10" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A10">
         <v>8</v>
       </c>
@@ -979,14 +1044,20 @@
       <c r="E10" s="4">
         <v>2.02</v>
       </c>
-      <c r="G10">
+      <c r="H10">
         <v>0.22600000000000001</v>
       </c>
-      <c r="H10">
+      <c r="I10">
         <v>0.94399999999999995</v>
       </c>
-    </row>
-    <row r="11" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="J10">
+        <v>0.23300000000000001</v>
+      </c>
+      <c r="K10">
+        <v>0.94</v>
+      </c>
+    </row>
+    <row r="11" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A11">
         <v>9</v>
       </c>
@@ -1002,14 +1073,20 @@
       <c r="E11" s="4">
         <v>2.08</v>
       </c>
-      <c r="G11">
+      <c r="H11">
         <v>0.22500000000000001</v>
       </c>
-      <c r="H11">
+      <c r="I11">
         <v>0.94599999999999995</v>
       </c>
-    </row>
-    <row r="12" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="J11">
+        <v>0.23599999999999999</v>
+      </c>
+      <c r="K11">
+        <v>0.93500000000000005</v>
+      </c>
+    </row>
+    <row r="12" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A12">
         <v>10</v>
       </c>
@@ -1025,14 +1102,20 @@
       <c r="E12" s="4">
         <v>2.0299999999999998</v>
       </c>
-      <c r="G12">
+      <c r="H12">
         <v>0.22600000000000001</v>
       </c>
-      <c r="H12">
+      <c r="I12">
         <v>0.94499999999999995</v>
       </c>
-    </row>
-    <row r="13" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="J12">
+        <v>0.23200000000000001</v>
+      </c>
+      <c r="K12">
+        <v>0.93600000000000005</v>
+      </c>
+    </row>
+    <row r="13" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A13">
         <v>12</v>
       </c>
@@ -1045,14 +1128,20 @@
       <c r="D13" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="G13">
+      <c r="H13">
         <v>0.39800000000000002</v>
       </c>
-      <c r="H13">
+      <c r="I13">
         <v>0.77900000000000003</v>
       </c>
-    </row>
-    <row r="14" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="J13">
+        <v>0.41599999999999998</v>
+      </c>
+      <c r="K13">
+        <v>0.75900000000000001</v>
+      </c>
+    </row>
+    <row r="14" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A14">
         <v>16</v>
       </c>
@@ -1068,14 +1157,20 @@
       <c r="E14" s="4">
         <v>2.0299999999999998</v>
       </c>
-      <c r="G14">
+      <c r="H14">
         <v>0.22700000000000001</v>
       </c>
-      <c r="H14">
+      <c r="I14">
         <v>0.94199999999999995</v>
       </c>
-    </row>
-    <row r="15" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="J14" s="4">
+        <v>0.23</v>
+      </c>
+      <c r="K14">
+        <v>0.94399999999999995</v>
+      </c>
+    </row>
+    <row r="15" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A15">
         <v>16</v>
       </c>
@@ -1091,14 +1186,20 @@
       <c r="E15" s="4">
         <v>2.1070000000000002</v>
       </c>
-      <c r="G15">
+      <c r="H15">
         <v>0.22700000000000001</v>
       </c>
-      <c r="H15">
+      <c r="I15">
         <v>0.93899999999999995</v>
       </c>
-    </row>
-    <row r="16" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="J15">
+        <v>0.23599999999999999</v>
+      </c>
+      <c r="K15">
+        <v>0.93400000000000005</v>
+      </c>
+    </row>
+    <row r="16" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A16">
         <v>16</v>
       </c>
@@ -1114,14 +1215,20 @@
       <c r="E16" s="4">
         <v>2.0419999999999998</v>
       </c>
-      <c r="G16">
+      <c r="H16">
         <v>0.22700000000000001</v>
       </c>
-      <c r="H16">
+      <c r="I16">
         <v>0.94099999999999995</v>
       </c>
-    </row>
-    <row r="17" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="J16">
+        <v>0.19900000000000001</v>
+      </c>
+      <c r="K16">
+        <v>0.97499999999999998</v>
+      </c>
+    </row>
+    <row r="17" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A17">
         <v>16</v>
       </c>
@@ -1137,14 +1244,20 @@
       <c r="E17" s="4">
         <v>2.02</v>
       </c>
-      <c r="G17">
+      <c r="H17">
         <v>0.22600000000000001</v>
       </c>
-      <c r="H17">
+      <c r="I17">
         <v>0.94299999999999995</v>
       </c>
-    </row>
-    <row r="18" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="J17">
+        <v>0.23599999999999999</v>
+      </c>
+      <c r="K17">
+        <v>0.93500000000000005</v>
+      </c>
+    </row>
+    <row r="18" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A18">
         <v>16</v>
       </c>
@@ -1160,14 +1273,20 @@
       <c r="E18" s="4">
         <v>2.0649999999999999</v>
       </c>
-      <c r="G18">
+      <c r="H18">
         <v>0.22700000000000001</v>
       </c>
-      <c r="H18">
+      <c r="I18">
         <v>0.94299999999999995</v>
       </c>
-    </row>
-    <row r="19" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="J18">
+        <v>0.23599999999999999</v>
+      </c>
+      <c r="K18">
+        <v>0.93500000000000005</v>
+      </c>
+    </row>
+    <row r="19" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A19">
         <v>16</v>
       </c>
@@ -1180,14 +1299,20 @@
       <c r="D19" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="G19">
+      <c r="H19">
         <v>0.443</v>
       </c>
-      <c r="H19">
+      <c r="I19">
         <v>0.73399999999999999</v>
       </c>
-    </row>
-    <row r="20" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="J19">
+        <v>0.46100000000000002</v>
+      </c>
+      <c r="K19">
+        <v>0.71599999999999997</v>
+      </c>
+    </row>
+    <row r="20" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A20">
         <v>16</v>
       </c>
@@ -1203,14 +1328,20 @@
       <c r="E20" s="4">
         <v>2.0870000000000002</v>
       </c>
-      <c r="G20">
+      <c r="H20">
         <v>0.224</v>
       </c>
-      <c r="H20">
+      <c r="I20">
         <v>0.99399999999999999</v>
       </c>
-    </row>
-    <row r="21" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="J20">
+        <v>0.23300000000000001</v>
+      </c>
+      <c r="K20">
+        <v>0.93799999999999994</v>
+      </c>
+    </row>
+    <row r="21" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A21">
         <v>16</v>
       </c>
@@ -1226,14 +1357,20 @@
       <c r="E21" s="4">
         <v>2.0390000000000001</v>
       </c>
-      <c r="G21">
+      <c r="H21">
         <v>0.22600000000000001</v>
       </c>
-      <c r="H21">
+      <c r="I21">
         <v>0.94299999999999995</v>
       </c>
-    </row>
-    <row r="22" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="J21">
+        <v>0.23799999999999999</v>
+      </c>
+      <c r="K21">
+        <v>0.93300000000000005</v>
+      </c>
+    </row>
+    <row r="22" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A22">
         <v>16</v>
       </c>
@@ -1249,14 +1386,20 @@
       <c r="E22" s="4">
         <v>2.09</v>
       </c>
-      <c r="G22">
+      <c r="H22">
         <v>0.22600000000000001</v>
       </c>
-      <c r="H22">
+      <c r="I22">
         <v>0.94099999999999995</v>
       </c>
-    </row>
-    <row r="23" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="J22">
+        <v>0.23899999999999999</v>
+      </c>
+      <c r="K22">
+        <v>0.93100000000000005</v>
+      </c>
+    </row>
+    <row r="23" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A23">
         <v>16</v>
       </c>
@@ -1272,14 +1415,20 @@
       <c r="E23" s="4">
         <v>2.0979999999999999</v>
       </c>
-      <c r="G23">
+      <c r="H23">
         <v>0.22500000000000001</v>
       </c>
-      <c r="H23">
+      <c r="I23">
         <v>0.94099999999999995</v>
       </c>
-    </row>
-    <row r="24" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="J23">
+        <v>0.23799999999999999</v>
+      </c>
+      <c r="K23">
+        <v>0.93300000000000005</v>
+      </c>
+    </row>
+    <row r="24" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A24">
         <v>16</v>
       </c>
@@ -1295,14 +1444,20 @@
       <c r="E24" s="4">
         <v>2.0859999999999999</v>
       </c>
-      <c r="G24">
+      <c r="H24">
         <v>0.22600000000000001</v>
       </c>
-      <c r="H24">
+      <c r="I24">
         <v>0.94199999999999995</v>
       </c>
-    </row>
-    <row r="25" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="J24">
+        <v>0.23699999999999999</v>
+      </c>
+      <c r="K24">
+        <v>0.93300000000000005</v>
+      </c>
+    </row>
+    <row r="25" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A25">
         <v>16</v>
       </c>
@@ -1315,11 +1470,17 @@
       <c r="D25" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="G25">
+      <c r="H25">
         <v>0.44500000000000001</v>
       </c>
-      <c r="H25">
+      <c r="I25">
         <v>0.73299999999999998</v>
+      </c>
+      <c r="J25">
+        <v>0.46100000000000002</v>
+      </c>
+      <c r="K25">
+        <v>0.71499999999999997</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Lab cattle slurry started
Started on extracted lab cattle slurry experiment - not done

Simply copied field-script, need to change experiment-specific constants
</commit_message>
<xml_diff>
--- a/Lab-trails/2026-01-06-cattle-slurry/2026-01-06-cattle-slurry-Picarro.xlsx
+++ b/Lab-trails/2026-01-06-cattle-slurry/2026-01-06-cattle-slurry-Picarro.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29530"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29725"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\mikae\Desktop\Github - speciale\Larsen-2025-Masterthesis-DFCs\Lab-trails\2026-01-06-cattle-slurry\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3E7A5DA6-C006-43C7-9BF5-9739F73E2725}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D6C09F16-E88A-470E-BCBB-02C6FCDED5BF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="360" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Jar and valve id overview" sheetId="1" r:id="rId1"/>
@@ -48,7 +48,8 @@
         <t>[Threaded comment]
 Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
 Comment:
-    Delayed by excacly 1 h from real time</t>
+    Real time noted
+09:17 in Picarro log-file, known delay by excatly 1 h</t>
       </text>
     </comment>
     <comment ref="I8" authorId="1" shapeId="0" xr:uid="{D6A11C27-28E7-4435-BC4A-E3E1711C9750}">
@@ -486,7 +487,8 @@
 <file path=xl/threadedComments/threadedComment1.xml><?xml version="1.0" encoding="utf-8"?>
 <ThreadedComments xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <threadedComment ref="F2" dT="2026-01-08T09:15:27.58" personId="{665E6C45-FDD8-469A-93B0-28134F14276F}" id="{DFE91DE2-97B6-4683-BB64-BFCD2C85D76D}">
-    <text>Delayed by excacly 1 h from real time</text>
+    <text>Real time noted
+09:17 in Picarro log-file, known delay by excatly 1 h</text>
   </threadedComment>
   <threadedComment ref="I8" dT="2026-01-08T09:23:24.74" personId="{665E6C45-FDD8-469A-93B0-28134F14276F}" id="{D6A11C27-28E7-4435-BC4A-E3E1711C9750}">
     <text>Didn’t write this, using an average from other jar measurements</text>

</xml_diff>

<commit_message>
Lab Cattle data treatment started
Inital extaction from DAT-files completed
Csv-file with PPB-data created
</commit_message>
<xml_diff>
--- a/Lab-trails/2026-01-06-cattle-slurry/2026-01-06-cattle-slurry-Picarro.xlsx
+++ b/Lab-trails/2026-01-06-cattle-slurry/2026-01-06-cattle-slurry-Picarro.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\mikae\Desktop\Github - speciale\Larsen-2025-Masterthesis-DFCs\Lab-trails\2026-01-06-cattle-slurry\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D6C09F16-E88A-470E-BCBB-02C6FCDED5BF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{818896A0-0BBC-4E32-B9CC-D772F47913E9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="2988" yWindow="2100" windowWidth="17280" windowHeight="8880" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Jar and valve id overview" sheetId="1" r:id="rId1"/>
@@ -1377,7 +1377,7 @@
         <v>16</v>
       </c>
       <c r="B22">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="C22">
         <v>18</v>

</xml_diff>